<commit_message>
convert all excel files to use relative links, update source files where necessary based on link validation script, convert all excel files into .xlsx format (from .xlsb), minor data updates based on corrected source files
</commit_message>
<xml_diff>
--- a/csv/model/CIMS_base/formula_CIMS_base_AB.xlsx
+++ b/csv/model/CIMS_base/formula_CIMS_base_AB.xlsx
@@ -1,171 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CIMS\dev\cims-models\csv\model\CIMS_base\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{36543896-C053-4CF5-BDDB-A404AE512B98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{14724549-7B89-4625-AD24-6A4785BB65F1}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId2"/>
   </externalReferences>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="29">
-  <si>
-    <t>&lt;-- Navigate by typing to search</t>
-  </si>
-  <si>
-    <t>Branch</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Region</t>
-  </si>
-  <si>
-    <t>Sector</t>
-  </si>
-  <si>
-    <t>Service</t>
-  </si>
-  <si>
-    <t>Technology</t>
-  </si>
-  <si>
-    <t>Parameter</t>
-  </si>
-  <si>
-    <t>Context</t>
-  </si>
-  <si>
-    <t>Sub_Context</t>
-  </si>
-  <si>
-    <t>Target</t>
-  </si>
-  <si>
-    <t>Source</t>
-  </si>
-  <si>
-    <t>Unit</t>
-  </si>
-  <si>
-    <t>Comments</t>
-  </si>
-  <si>
-    <t>CIMS.CAN</t>
-  </si>
-  <si>
-    <t>CAN</t>
-  </si>
-  <si>
-    <t>Service requested</t>
-  </si>
-  <si>
-    <t>CIMS.CAN.AB</t>
-  </si>
-  <si>
-    <t>n/a</t>
-  </si>
-  <si>
-    <t>unit</t>
-  </si>
-  <si>
-    <t>AB</t>
-  </si>
-  <si>
-    <t>Service provided</t>
-  </si>
-  <si>
-    <t>Competition type</t>
-  </si>
-  <si>
-    <t>Attribute</t>
-  </si>
-  <si>
-    <t>Population</t>
-  </si>
-  <si>
-    <t>StatCan</t>
-  </si>
-  <si>
-    <t>persons</t>
-  </si>
-  <si>
-    <t>GDP</t>
-  </si>
-  <si>
-    <t>$ million</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -184,30 +49,86 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
+<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook r:id="rId1">
     <sheetNames>
       <sheetName val="Control"/>
       <sheetName val="Macro"/>
@@ -5101,311 +5022,405 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{103DF7E6-4D3C-405A-9F8E-2718AFE29276}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:X7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
-        <v>0</v>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>&lt;-- Navigate by typing to search</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Context</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Sub_Context</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="N2" t="n">
+        <v>2005</v>
+      </c>
+      <c r="O2" t="n">
+        <v>2010</v>
+      </c>
+      <c r="P2" t="n">
+        <v>2015</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="R2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="S2" t="n">
+        <v>2030</v>
+      </c>
+      <c r="T2" t="n">
+        <v>2035</v>
+      </c>
+      <c r="U2" t="n">
+        <v>2040</v>
+      </c>
+      <c r="V2" t="n">
+        <v>2045</v>
+      </c>
+      <c r="W2" t="n">
+        <v>2050</v>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CIMS.CAN</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CAN</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Service requested</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>CIMS.CAN.AB</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H2" t="s">
-        <v>8</v>
-      </c>
-      <c r="I2" t="s">
-        <v>9</v>
-      </c>
-      <c r="J2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K2" t="s">
-        <v>11</v>
-      </c>
-      <c r="L2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M2">
-        <v>2000</v>
-      </c>
-      <c r="N2">
-        <v>2005</v>
-      </c>
-      <c r="O2">
-        <v>2010</v>
-      </c>
-      <c r="P2">
-        <v>2015</v>
-      </c>
-      <c r="Q2">
-        <v>2020</v>
-      </c>
-      <c r="R2">
-        <v>2025</v>
-      </c>
-      <c r="S2">
-        <v>2030</v>
-      </c>
-      <c r="T2">
-        <v>2035</v>
-      </c>
-      <c r="U2">
-        <v>2040</v>
-      </c>
-      <c r="V2">
-        <v>2045</v>
-      </c>
-      <c r="W2">
-        <v>2050</v>
-      </c>
-      <c r="X2" t="s">
-        <v>13</v>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S3" t="n">
+        <v>1</v>
+      </c>
+      <c r="T3" t="n">
+        <v>1</v>
+      </c>
+      <c r="U3" t="n">
+        <v>1</v>
+      </c>
+      <c r="V3" t="n">
+        <v>1</v>
+      </c>
+      <c r="W3" t="n">
+        <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J3" t="s">
-        <v>17</v>
-      </c>
-      <c r="K3" t="s">
-        <v>18</v>
-      </c>
-      <c r="L3" t="s">
-        <v>19</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-      <c r="N3">
-        <v>1</v>
-      </c>
-      <c r="O3">
-        <v>1</v>
-      </c>
-      <c r="P3">
-        <v>1</v>
-      </c>
-      <c r="Q3">
-        <v>1</v>
-      </c>
-      <c r="R3">
-        <v>1</v>
-      </c>
-      <c r="S3">
-        <v>1</v>
-      </c>
-      <c r="T3">
-        <v>1</v>
-      </c>
-      <c r="U3">
-        <v>1</v>
-      </c>
-      <c r="V3">
-        <v>1</v>
-      </c>
-      <c r="W3">
-        <v>1</v>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CIMS.CAN.AB</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Service provided</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" t="s">
-        <v>21</v>
-      </c>
-      <c r="L4" t="s">
-        <v>19</v>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CIMS.CAN.AB</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Competition type</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" t="s">
-        <v>3</v>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CIMS.CAN.AB</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>StatCan</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>persons</t>
+        </is>
+      </c>
+      <c r="M6">
+        <f t="array" ref="M6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(M$2,[1]!CIMS_year))</f>
+        <v/>
+      </c>
+      <c r="N6">
+        <f t="array" ref="N6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(N$2,[1]!CIMS_year))</f>
+        <v/>
+      </c>
+      <c r="O6">
+        <f t="array" ref="O6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(O$2,[1]!CIMS_year))</f>
+        <v/>
+      </c>
+      <c r="P6">
+        <f t="array" ref="P6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(P$2,[1]!CIMS_year))</f>
+        <v/>
+      </c>
+      <c r="Q6">
+        <f t="array" ref="Q6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(Q$2,[1]!CIMS_year))</f>
+        <v/>
+      </c>
+      <c r="R6">
+        <f t="array" ref="R6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(R$2,[1]!CIMS_year))</f>
+        <v/>
+      </c>
+      <c r="S6">
+        <f t="array" ref="S6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(S$2,[1]!CIMS_year))</f>
+        <v/>
+      </c>
+      <c r="T6">
+        <f t="array" ref="T6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(T$2,[1]!CIMS_year))</f>
+        <v/>
+      </c>
+      <c r="U6">
+        <f t="array" ref="U6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(U$2,[1]!CIMS_year))</f>
+        <v/>
+      </c>
+      <c r="V6">
+        <f t="array" ref="V6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(V$2,[1]!CIMS_year))</f>
+        <v/>
+      </c>
+      <c r="W6">
+        <f t="array" ref="W6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(W$2,[1]!CIMS_year))</f>
+        <v/>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" t="s">
-        <v>20</v>
-      </c>
-      <c r="G6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L6" t="s">
-        <v>26</v>
-      </c>
-      <c r="M6" cm="1">
-        <f t="array" ref="M6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(M$2,[1]!CIMS_year))</f>
-        <v>3004198</v>
-      </c>
-      <c r="N6" cm="1">
-        <f t="array" ref="N6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(N$2,[1]!CIMS_year))</f>
-        <v>3321768</v>
-      </c>
-      <c r="O6" cm="1">
-        <f t="array" ref="O6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(O$2,[1]!CIMS_year))</f>
-        <v>3732082</v>
-      </c>
-      <c r="P6" cm="1">
-        <f t="array" ref="P6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(P$2,[1]!CIMS_year))</f>
-        <v>4144491</v>
-      </c>
-      <c r="Q6" cm="1">
-        <f t="array" ref="Q6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(Q$2,[1]!CIMS_year))</f>
-        <v>4420029</v>
-      </c>
-      <c r="R6" cm="1">
-        <f t="array" ref="R6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(R$2,[1]!CIMS_year))</f>
-        <v>4965000</v>
-      </c>
-      <c r="S6" cm="1">
-        <f t="array" ref="S6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(S$2,[1]!CIMS_year))</f>
-        <v>5460100</v>
-      </c>
-      <c r="T6" cm="1">
-        <f t="array" ref="T6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(T$2,[1]!CIMS_year))</f>
-        <v>5976700</v>
-      </c>
-      <c r="U6" cm="1">
-        <f t="array" ref="U6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(U$2,[1]!CIMS_year))</f>
-        <v>6515600</v>
-      </c>
-      <c r="V6" cm="1">
-        <f t="array" ref="V6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(V$2,[1]!CIMS_year))</f>
-        <v>6751778.2937559607</v>
-      </c>
-      <c r="W6" cm="1">
-        <f t="array" ref="W6">INDEX([1]!CIMS_population,_xlfn.XMATCH($C6,[1]!region_CIMS),_xlfn.XMATCH(W$2,[1]!CIMS_year))</f>
-        <v>6981842.726861191</v>
-      </c>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" t="s">
-        <v>23</v>
-      </c>
-      <c r="H7" t="s">
-        <v>27</v>
-      </c>
-      <c r="K7" t="s">
-        <v>25</v>
-      </c>
-      <c r="L7" t="s">
-        <v>28</v>
-      </c>
-      <c r="M7" cm="1">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CIMS.CAN.AB</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>GDP</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>StatCan</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>$ million</t>
+        </is>
+      </c>
+      <c r="M7">
         <f t="array" ref="M7">INDEX([1]!CIMS_GDP,_xlfn.XMATCH($C7,[1]!region_CIMS),_xlfn.XMATCH(M$2,[1]!CIMS_year))</f>
-        <v>241251.75158053398</v>
-      </c>
-      <c r="N7" cm="1">
+        <v/>
+      </c>
+      <c r="N7">
         <f t="array" ref="N7">INDEX([1]!CIMS_GDP,_xlfn.XMATCH($C7,[1]!region_CIMS),_xlfn.XMATCH(N$2,[1]!CIMS_year))</f>
-        <v>286047.23224697507</v>
-      </c>
-      <c r="O7" cm="1">
+        <v/>
+      </c>
+      <c r="O7">
         <f t="array" ref="O7">INDEX([1]!CIMS_GDP,_xlfn.XMATCH($C7,[1]!region_CIMS),_xlfn.XMATCH(O$2,[1]!CIMS_year))</f>
-        <v>311884.83832539228</v>
-      </c>
-      <c r="P7" cm="1">
+        <v/>
+      </c>
+      <c r="P7">
         <f t="array" ref="P7">INDEX([1]!CIMS_GDP,_xlfn.XMATCH($C7,[1]!region_CIMS),_xlfn.XMATCH(P$2,[1]!CIMS_year))</f>
-        <v>371864.0496689151</v>
-      </c>
-      <c r="Q7" cm="1">
+        <v/>
+      </c>
+      <c r="Q7">
         <f t="array" ref="Q7">INDEX([1]!CIMS_GDP,_xlfn.XMATCH($C7,[1]!region_CIMS),_xlfn.XMATCH(Q$2,[1]!CIMS_year))</f>
-        <v>352708.69722059922</v>
-      </c>
-      <c r="R7" cm="1">
+        <v/>
+      </c>
+      <c r="R7">
         <f t="array" ref="R7">INDEX([1]!CIMS_GDP,_xlfn.XMATCH($C7,[1]!region_CIMS),_xlfn.XMATCH(R$2,[1]!CIMS_year))</f>
-        <v>398094.70776005066</v>
-      </c>
-      <c r="S7" cm="1">
+        <v/>
+      </c>
+      <c r="S7">
         <f t="array" ref="S7">INDEX([1]!CIMS_GDP,_xlfn.XMATCH($C7,[1]!region_CIMS),_xlfn.XMATCH(S$2,[1]!CIMS_year))</f>
-        <v>440960.56814001396</v>
-      </c>
-      <c r="T7" cm="1">
+        <v/>
+      </c>
+      <c r="T7">
         <f t="array" ref="T7">INDEX([1]!CIMS_GDP,_xlfn.XMATCH($C7,[1]!region_CIMS),_xlfn.XMATCH(T$2,[1]!CIMS_year))</f>
-        <v>484955.42138564883</v>
-      </c>
-      <c r="U7" cm="1">
+        <v/>
+      </c>
+      <c r="U7">
         <f t="array" ref="U7">INDEX([1]!CIMS_GDP,_xlfn.XMATCH($C7,[1]!region_CIMS),_xlfn.XMATCH(U$2,[1]!CIMS_year))</f>
-        <v>535701.75694266777</v>
-      </c>
-      <c r="V7" cm="1">
+        <v/>
+      </c>
+      <c r="V7">
         <f t="array" ref="V7">INDEX([1]!CIMS_GDP,_xlfn.XMATCH($C7,[1]!region_CIMS),_xlfn.XMATCH(V$2,[1]!CIMS_year))</f>
-        <v>591527.46226970514</v>
-      </c>
-      <c r="W7" cm="1">
+        <v/>
+      </c>
+      <c r="W7">
         <f t="array" ref="W7">INDEX([1]!CIMS_GDP,_xlfn.XMATCH($C7,[1]!region_CIMS),_xlfn.XMATCH(W$2,[1]!CIMS_year))</f>
-        <v>650318.67160160968</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update parameter names, code variable names to align with params, change no_ineritable to inheritable and switch default from FALSE to TRUE, clarify 'market share' to be 'market_share_total' in csv files and 'market_share_new' in tech competitions and update code accordingly, remove 'tech compete' hard coded instead reference list.py
</commit_message>
<xml_diff>
--- a/csv/model/CIMS_base/formula_CIMS_base_AB.xlsx
+++ b/csv/model/CIMS_base/formula_CIMS_base_AB.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3624" yWindow="2148" windowWidth="17280" windowHeight="8880" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,7 +12,7 @@
     <externalReference r:id="rId2"/>
   </externalReferences>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1" calcOnSave="0"/>
 </workbook>
 </file>
 
@@ -139,6 +139,7 @@
       <sheetName val="CER"/>
       <sheetName val="Conversions"/>
       <sheetName val="Coefficients"/>
+      <sheetName val="macro inputs"/>
     </sheetNames>
     <definedNames>
       <definedName name="CIMS_GDP" refersTo="='Macro'!$D$59:$R$74"/>
@@ -1706,39 +1707,6 @@
           <cell r="D1" t="str">
             <v>Sector</v>
           </cell>
-          <cell r="E1" t="str">
-            <v>Fuel</v>
-          </cell>
-          <cell r="F1" t="str">
-            <v>Unit</v>
-          </cell>
-          <cell r="I1" t="str">
-            <v>Source</v>
-          </cell>
-          <cell r="K1">
-            <v>2000</v>
-          </cell>
-          <cell r="L1">
-            <v>2005</v>
-          </cell>
-          <cell r="M1">
-            <v>2010</v>
-          </cell>
-          <cell r="N1">
-            <v>2015</v>
-          </cell>
-          <cell r="O1">
-            <v>2021</v>
-          </cell>
-          <cell r="P1">
-            <v>2025</v>
-          </cell>
-          <cell r="Q1">
-            <v>2030</v>
-          </cell>
-          <cell r="R1">
-            <v>2035</v>
-          </cell>
         </row>
         <row r="26">
           <cell r="B26" t="str">
@@ -2460,18 +2428,6 @@
           <cell r="D1" t="str">
             <v>Sector</v>
           </cell>
-          <cell r="E1" t="str">
-            <v>Context</v>
-          </cell>
-          <cell r="F1" t="str">
-            <v>Sub_context</v>
-          </cell>
-          <cell r="G1" t="str">
-            <v>Unit</v>
-          </cell>
-          <cell r="J1" t="str">
-            <v>Source</v>
-          </cell>
         </row>
         <row r="24">
           <cell r="B24" t="str">
@@ -2489,39 +2445,6 @@
           <cell r="D1" t="str">
             <v>Sector</v>
           </cell>
-          <cell r="E1" t="str">
-            <v>Fuel</v>
-          </cell>
-          <cell r="F1" t="str">
-            <v>Unit</v>
-          </cell>
-          <cell r="I1" t="str">
-            <v>Source</v>
-          </cell>
-          <cell r="K1">
-            <v>2000</v>
-          </cell>
-          <cell r="L1">
-            <v>2005</v>
-          </cell>
-          <cell r="M1">
-            <v>2010</v>
-          </cell>
-          <cell r="N1">
-            <v>2015</v>
-          </cell>
-          <cell r="O1">
-            <v>2020</v>
-          </cell>
-          <cell r="P1">
-            <v>2025</v>
-          </cell>
-          <cell r="Q1">
-            <v>2030</v>
-          </cell>
-          <cell r="R1">
-            <v>2035</v>
-          </cell>
         </row>
         <row r="59">
           <cell r="D59" t="str">
@@ -3134,45 +3057,6 @@
           <cell r="D1" t="str">
             <v>Commercial</v>
           </cell>
-          <cell r="E1" t="str">
-            <v>Industrial</v>
-          </cell>
-          <cell r="G1">
-            <v>2000</v>
-          </cell>
-          <cell r="H1">
-            <v>2001</v>
-          </cell>
-          <cell r="I1">
-            <v>2002</v>
-          </cell>
-          <cell r="J1">
-            <v>2003</v>
-          </cell>
-          <cell r="K1">
-            <v>2004</v>
-          </cell>
-          <cell r="L1">
-            <v>2005</v>
-          </cell>
-          <cell r="M1">
-            <v>2006</v>
-          </cell>
-          <cell r="N1">
-            <v>2007</v>
-          </cell>
-          <cell r="O1">
-            <v>2008</v>
-          </cell>
-          <cell r="P1">
-            <v>2009</v>
-          </cell>
-          <cell r="Q1">
-            <v>2010</v>
-          </cell>
-          <cell r="R1">
-            <v>2011</v>
-          </cell>
         </row>
         <row r="59">
           <cell r="D59">
@@ -3292,33 +3176,6 @@
           <cell r="D1" t="str">
             <v>Sector</v>
           </cell>
-          <cell r="E1" t="str">
-            <v>Fuel</v>
-          </cell>
-          <cell r="F1" t="str">
-            <v>Unit</v>
-          </cell>
-          <cell r="I1" t="str">
-            <v>Source</v>
-          </cell>
-          <cell r="K1" t="str">
-            <v>Unit</v>
-          </cell>
-          <cell r="N1">
-            <v>1995</v>
-          </cell>
-          <cell r="O1">
-            <v>1996</v>
-          </cell>
-          <cell r="P1">
-            <v>1997</v>
-          </cell>
-          <cell r="Q1">
-            <v>1998</v>
-          </cell>
-          <cell r="R1">
-            <v>1999</v>
-          </cell>
         </row>
         <row r="26">
           <cell r="B26" t="str">
@@ -3968,9 +3825,6 @@
           <cell r="D1" t="str">
             <v>To</v>
           </cell>
-          <cell r="G1" t="str">
-            <v>Multiply by</v>
-          </cell>
         </row>
       </sheetData>
       <sheetData sheetId="8">
@@ -3978,45 +3832,6 @@
           <cell r="D1" t="str">
             <v>For prices</v>
           </cell>
-          <cell r="F1" t="str">
-            <v>Source</v>
-          </cell>
-          <cell r="G1">
-            <v>2000</v>
-          </cell>
-          <cell r="H1">
-            <v>2001</v>
-          </cell>
-          <cell r="I1">
-            <v>2002</v>
-          </cell>
-          <cell r="J1">
-            <v>2003</v>
-          </cell>
-          <cell r="K1">
-            <v>2004</v>
-          </cell>
-          <cell r="L1">
-            <v>2005</v>
-          </cell>
-          <cell r="M1">
-            <v>2006</v>
-          </cell>
-          <cell r="N1">
-            <v>2007</v>
-          </cell>
-          <cell r="O1">
-            <v>2008</v>
-          </cell>
-          <cell r="P1">
-            <v>2009</v>
-          </cell>
-          <cell r="Q1">
-            <v>2010</v>
-          </cell>
-          <cell r="R1">
-            <v>2011</v>
-          </cell>
         </row>
         <row r="19">
           <cell r="B19" t="str">
@@ -4701,6 +4516,7 @@
           </cell>
         </row>
       </sheetData>
+      <sheetData sheetId="9" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -5023,12 +4839,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+  <sheetPr codeName="Sheet1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:X7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
@@ -5155,7 +4971,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Service requested</t>
+          <t>service_request</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -5225,7 +5041,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Service provided</t>
+          <t>service_provide</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -5252,7 +5068,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Competition type</t>
+          <t>competition</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -5279,7 +5095,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Attribute</t>
+          <t>attribute</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -5360,7 +5176,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Attribute</t>
+          <t>attribute</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">

</xml_diff>